<commit_message>
Se quita la seccion de presupuesto, pues es innecesaria y redundante
</commit_message>
<xml_diff>
--- a/static/assets/plantilla.xlsx
+++ b/static/assets/plantilla.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movimientos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38,8 +38,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D3D3D3"/>
-        <bgColor rgb="00D3D3D3"/>
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -423,12 +422,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -457,52 +452,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Ejemplo ingreso</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>ingreso</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-07-02</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Mercado quincena</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Alimentación</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>120000</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>gasto</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>